<commit_message>
enemies.xlsx: real biology, citations, Sentinel (mast cell)
Restructured sheet: Description replaced with Real Biology
(factual cell/molecule descriptions), Citation (key paper),
and Wikipedia link for each entity. Added Sentinel (mast cell
sniper: fixed position, cone watch, direct shot, cover-based
counterplay). Dropped Sporadic and Spitter designs (too much
area denial overlap). 13 lethal enemies, 5 hazards, 11
ecosystem interactions across 3 sheets.
</commit_message>
<xml_diff>
--- a/to-rust-as-we-fall/data/enemies.xlsx
+++ b/to-rust-as-we-fall/data/enemies.xlsx
@@ -438,18 +438,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,35 +466,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Real Biology</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Citation</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Detection</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>States</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Attack/Mechanic</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Zones</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Counters</t>
         </is>
@@ -512,35 +518,40 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Catechol-type siderophore (bacterial iron scavenger)</t>
+          <t>Catechol-type siderophore (e.g. enterobactin). Small-molecule iron chelators secreted by bacteria to scavenge ferric iron (Fe3+) from the host. Catecholates are the highest-affinity class, outcompeting host transferrin and lactoferrin. In CNS infection, siderophore-mediated iron piracy exacerbates the labile iron pool, fueling oxidative damage.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Ring-shaped, compact, fist-sized. Six articulated legs. Dull iron-brown carapace with geometric vein patterning. Most common early-game siderophore.</t>
+          <t>Kramer et al. (2020) Nature Reviews Microbiology, "Bacterial siderophores in community and host interactions." 18(3), 152–163.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Siderophore</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Iron gradient sensing. Attracted to iron-rich characters (Myke, Oli) and iron blooms. No visual/sound detection.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>idle, foraging, pursue, investigate, search, scatter, feeding, satiated</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Iron drain (HP + Oli reserves). Reproduces at iron bloom zones.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Zone 2-3. 90% of early siderophores.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Myke fire, Amoebae engulf, clear iron blooms</t>
         </is>
@@ -559,35 +570,40 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pyoverdine-type siderophore (fluorescent iron chelator)</t>
+          <t>Pyoverdine-type siderophore (carboxylate class). Fluorescent yellow-green iron chelator produced by Pseudomonas species. Pyoverdine is both a virulence factor and a signaling molecule that regulates toxin production. Its fluorescence under UV is diagnostically distinctive.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Elongated teardrop. Yellow-green fluorescent glow, semi-translucent. Thrives near moisture and breaches.</t>
+          <t>Kramer et al. (2020) Nature Reviews Microbiology, "Bacterial siderophores in community and host interactions." 18(3), 152–163.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Pyoverdine</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Iron gradient sensing. Same as Chelator.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>idle, foraging, pursue, investigate, search, scatter, feeding, satiated</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Iron drain. Increases near breach areas.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Zone 2-3. Increases mid-game near breaches, dominant late game.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Myke fire, Amoebae engulf</t>
         </is>
@@ -606,35 +622,40 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hydroxamate-type siderophore (chain-linked iron binder)</t>
+          <t>Hydroxamate-type siderophore (e.g. desferrioxamine). Produced by Streptomyces and other soil bacteria. Hydroxamates form stable 1:1 complexes with Fe3+ via hydroxamic acid groups. Desferrioxamine is used clinically as an iron chelator (Desferal) for iron overload conditions, demonstrating the potency of this chelation mechanism.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Long segmented worm. Moves like dragged chains. Camouflages as pipes/conduits. Moves through cracks and vents.</t>
+          <t>Kramer et al. (2020) Nature Reviews Microbiology, "Bacterial siderophores in community and host interactions." 18(3), 152–163.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Desferrioxamine</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Iron gradient sensing. Same as Chelator.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>idle, foraging, pursue, investigate, search, scatter, feeding, satiated</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Iron drain. Segmented body — lead point + trailing segments with spring-damped follow. Anchor constraint limits reach. All segments deal contact damage.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Zone 2-3. Everywhere late game.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Myke fire, Amoebae engulf, sever from anchor</t>
         </is>
@@ -653,35 +674,40 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mycobactin-type siderophore (surface biofilm iron extractor)</t>
+          <t>Mycobactin-type siderophore (mixed-type, lipophilic). Produced by Mycobacterium species including M. tuberculosis. Mycobactins are membrane-associated, extracting iron at the cell surface rather than being secreted into the environment. This makes them sessile iron extractors that operate by direct contact with iron-containing substrates.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Living biofilm patches on infrastructure surfaces. Spreads slowly. Passive iron drain via filaments.</t>
+          <t>Kramer et al. (2020) Nature Reviews Microbiology, "Bacterial siderophores in community and host interactions." 18(3), 152–163.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Mycobactin</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Passive — does not pursue. Spreads along surfaces.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>spreading, dormant</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Passive iron drain on contact. Area denial. Spreads if unaddressed.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Zone 2-3. Accumulates on unmaintained surfaces.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Peris flora tending, Myke fire</t>
         </is>
@@ -700,35 +726,40 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Opportunistic pathogens that establish biofilms and transform environments</t>
+          <t>Based on opportunistic pathogens (e.g. P. gingivalis, Candida) that establish biofilms in the CNS. Biofilms are structured microbial communities encased in extracellular polymeric substance (EPS), conferring up to 1000-fold antibiotic resistance. Amyloid-beta itself may function as an antimicrobial peptide that entraps pathogens in biofilm-like plaques. Polymicrobial biofilms have been detected in Alzheimer's brain tissue.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Large, slow, rooted growths. Fuse with infrastructure. Early scouts more mobile than mature colonies.</t>
+          <t>Kumar et al. (2016) Science Translational Medicine, "Amyloid-beta peptide protects against microbial infection in mouse and worm models of Alzheimer's disease." 8(340), 340ra72.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Biofilm</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Environmental conditions (humidity, temperature, barrier integrity). Drawn to environmental failure.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>scouting, anchoring (vulnerable), colonized, spreading</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Changes iron distribution, redirects siderophore patrols. Area denial: slow movement, stamina drain, perception interference. Blocks Naturalizer patrols (creates safe pockets).</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Zone 2-3. Spread increases over time if unmanaged.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Peris flora (slow, permanent), Myke Inferno (fast, temporary). Clear scouts early.</t>
         </is>
@@ -747,37 +778,42 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Intracellular pathogens that hijack cellular machinery</t>
+          <t>Based on intracellular pathogens that hijack host cell machinery (e.g. Chlamydia pneumoniae, HSV-1, Toxoplasma gondii). These organisms survive and replicate within neurons and glia by subverting endosomal trafficking, autophagy, and immune signaling. Persistent intracellular infection triggers chronic low-grade inflammation, amyloid-beta deposition (proposed as antimicrobial response), and progressive neurodegeneration.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Medium-sized, fast, almost humanoid but uncanny. Moves too smoothly, proportions subtly wrong, unnatural sheen.</t>
+          <t>Readhead et al. (2018) Neuron, "Multiscale Analysis of Independent Alzheimer's Cohorts Finds Disruption of Molecular, Genetic, and Clinical Networks by Human Herpesvirus." 99(1), 64–82.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Intracellular_parasite</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Sight and sound. Visual detection cone on Aster overlay. Responds to running, ability use, combat sounds.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>stalking, alerted, pursuing, capturing, returning</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Capture grapple (not instant death). Captured characters immobilized, take damage over time. Dragged off-screen = rescue mission from nest. Faster than walk, slower than run.</t>
-        </is>
-      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>Capture grapple (not instant death). Captured characters immobilized, take damage over time. Dragged off-screen = rescue mission. Faster than walk, slower than run.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>Zone 3 patrols. Avoids Infiltrator colonies.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Move quietly, scout patrol routes, time movement windows. Other party members can interrupt grapple.</t>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Move quietly, scout patrol routes, time movement windows. Party members can interrupt grapple.</t>
         </is>
       </c>
     </row>
@@ -794,35 +830,40 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Free-living amoebae (Naegleria, Acanthamoeba). Single-celled phagocytic organisms.</t>
+          <t>Based on free-living amoebae (Naegleria fowleri, Acanthamoeba). N. fowleri causes primary amoebic meningoencephalitis (PAM), migrating along the olfactory nerve to the brain. Both species destroy brain tissue through contact-dependent trogocytosis (nibbling phagocytosis), pore-forming proteins (naegleriapores), and secreted proteases. They also serve as environmental reservoirs for intracellular bacteria.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Translucent shifting blobs with overlapping circular membranes. Pulsing movement. Brownish-amber, brightens to yellow-amber when pursuing.</t>
+          <t>Moseman, E.A. (2020) PLoS Pathogens, "The ins and outs of Naegleria infection." 16(10), e1008857.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Naegleria_fowleri</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Senses anything living within ~6 tiles. Biased toward iron blooms when idle. Cannot sense through doors.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>roaming, pursuing, engulfing, digesting, attacking</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Engulfs siderophores over ~3s (both freeze). Contact damage comparable to siderophore drain. Ecosystem role: natural population control.</t>
-        </is>
-      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>Engulfs siderophores over ~3s (both freeze). Contact damage comparable to siderophore drain. Ecosystem role: natural siderophore population control.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>Zone 2-3 iron-rich corridors.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Avoid — they thin siderophore populations naturally. Use as ecological tool.</t>
         </is>
@@ -841,37 +882,42 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Gingipain cysteine proteases from P. gingivalis. Degrade structural proteins (tau, cytoskeleton). Found in 90%+ postmortem AD brains.</t>
+          <t>Based on gingipain cysteine proteases from Porphyromonas gingivalis. Gingipains (Kgp, RgpA, RgpB) degrade host proteins including immunoglobulins, complement factors, and structural proteins like tau. Detected in over 90% of examined Alzheimer's brain samples, with levels correlating to tau and ubiquitin pathology burden. A gingipain inhibitor (COR388) reduced bacterial load and neurodegeneration in mouse models.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Elongated, low-slung, fast. Two vibrating mandibles. Dark red-brown carapace. Six legs. Moves like centipede, climbs walls, drops from ceilings. Hunt in pairs/trios.</t>
+          <t>Dominy et al. (2019) Science Advances, "Porphyromonas gingivalis in Alzheimer's disease brains: Evidence for disease causation and treatment with small-molecule inhibitors." 5(1), eaau3333.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Gingipain</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Metabolic signatures (protein/metabolic activity). Pursue strongest signal in range. Attracted to ability use.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>idle, pursuit</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Latch and drain stamina (not HP). At zero stamina, drain ATP. Dodge roll detaches but costs stamina (self-defeating loop).</t>
-        </is>
-      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>Latch and drain stamina (not HP). At zero stamina, drain ATP. Dodge roll detaches but costs stamina (self-defeating). Hunt in pairs/trios. Climb walls, drop from ceilings.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>Zone 2-3. Sparse in maintained areas, dense in degraded zones.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Myke fire (instant detach), Tyreg shot, physical attack. Leave some siderophores alive as distraction targets.</t>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Myke fire (instant detach), Tyreg shot, physical attack. Leave some siderophores alive as distraction.</t>
         </is>
       </c>
     </row>
@@ -888,35 +934,40 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Neutrophils. First-response immune cells that release destructive enzymes indiscriminately.</t>
+          <t>Based on neutrophils, the most abundant circulating granulocytes and first innate immune responders. Kill pathogens through phagocytosis, degranulation (myeloperoxidase, elastase, defensins), and neutrophil extracellular traps (NETs). In AD, neutrophils infiltrate brain parenchyma through compromised BBB and are found adhered to cortical vessels and within amyloid plaque-bearing regions, where their proteases and ROS cause collateral neuronal damage.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Compact, spherical, pale blue-white with granular bumps. Multiple pseudopods. Slightly translucent with visible multi-lobed nucleus. Arrive in packs of 3-5.</t>
+          <t>Zenaro et al. (2015) Nature Medicine, "Neutrophils promote Alzheimer's disease-like pathology and cognitive decline via LFA-1 integrin." 21(8), 880–886.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Neutrophil</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Combat and damage events (not characters directly). Home in on damage sites.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>converging, degranulating</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Degranulation: radial enzyme burst damaging everything in radius (no friend/foe distinction). Triggered by damage signals.</t>
-        </is>
-      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>Degranulation: radial enzyme burst damaging everything in radius (no friend/foe distinction). Arrive in packs of 3-5. Triggered by damage signals.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>Zone 2-3. Dense near Infiltrator colonies, combat sites. Sparse in Dead Zones.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>End fights fast and quiet. Tyreg sidearm = low signal. Myke Inferno = massive signal = catastrophic escalation.</t>
         </is>
@@ -935,35 +986,40 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Complement cascade proteins. Molecular missiles that punch holes in cell membranes (MAC formation).</t>
+          <t>Based on the complement cascade membrane attack complex (MAC, C5b-9). The complement system is ~30 plasma proteins that tag pathogens (opsonization via C3b), recruit immune cells (anaphylatoxins C3a, C5a), and directly lyse targets through MAC pore formation. In the brain, C1q and C3 tag synapses for elimination by microglia (complement-mediated synaptic pruning), pathologically reactivated in AD, causing excessive synapse loss.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Cluster of interlocking geometric shapes assembling mid-air over ~0.5s (warning window). Pale crystalline projectile trailing faint shimmer. Fragments on impact.</t>
+          <t>Hong et al. (2016) Science, "Complement and microglia mediate early synapse loss in Alzheimer mouse models." 352(6286), 712–716.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Complement_membrane_attack_complex</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Not independent — triggered by Naturalizer tag-flagging, Responder degranulation, immune-activation sites.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>assembling (0.5s warning), projectile (straight-line, very fast, no turning)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Significant burst damage. Fragmentation deals secondary AoE. Miss if target moves. Multiple can trigger simultaneously.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Zone 2 (common, Checkpoint Plazas dense). Rare in deep Zone 3. Absent in Dead Zones.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Oli Barrier (blocks), Peris Wrap (absorbs), Tyreg shoot mid-flight, perpendicular dodge roll.</t>
         </is>
@@ -982,35 +1038,40 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Natural Killer (NK) cells. Innate immune cells that kill without prior sensitization. Check MHC-I presentation.</t>
+          <t>Based on Natural Killer (NK) cells, cytotoxic innate lymphocytes that survey for cells with reduced MHC-I expression ("missing self" hypothesis). Kill targets through perforin/granzyme exocytosis. In AD brains, NK cells can directly kill neurons and neural progenitor cells; depletion in mouse models improved cognitive outcomes. They modulate neuroinflammation through IFN-gamma and TNF-alpha secretion.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Clean uniforms, neutral colors, clinical movement. Pairs or trios with synchronized spacing. Carry handheld scanners. Look like trustworthy staff.</t>
+          <t>Zhang et al. (2020) Cell Reports, "Depletion of NK Cells Improves Cognitive Function in the Alzheimer Disease Mouse Model." 33(12), 108516.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Natural_killer_cell</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Tag-scanning (electromagnetic/biochemical). Coherent tags = invisible. Degrading tags = increasing detection range. Myke (no tag) = always triggers.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>patrol, alert, containment, returning</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Active scans have longer range. Confirmed detection = radio support + calm coordinated containment. Removal = incapacitation (rescue from processing station).</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Zone 2 Transit Corridors and Checkpoint Plazas. Routine schedules.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Tyreg immune balancing (suppresses scan sensitivity). Learn patrol routes. Route Peris through NK-free zones.</t>
         </is>
@@ -1029,37 +1090,94 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Peripheral neutrophils crossing failing blood-brain barrier during sleep (increased BBB permeability).</t>
+          <t>Based on peripheral neutrophils crossing the failing blood-brain barrier. The BBB is a selectively permeable endothelial structure; breakdown is an early biomarker of cognitive decline, beginning in the hippocampus. Pericyte degeneration drives increased permeability, allowing peripheral immune cells, fibrinogen, and plasma proteins to infiltrate the parenchyma. BBB permeability fluctuates diurnally, with increased transport during sleep.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Glow red in darkness. Fast, destructive, indiscriminate. Spawn far from characters at nightfall. Cannot enter shelters but circle them.</t>
+          <t>Nation et al. (2019) Nature Medicine, "Blood-brain barrier breakdown is an early biomarker of human cognitive dysfunction." 25(2), 270–276.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Blood%E2%80%93brain_barrier</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Inflammatory signals through doors (chemical gradient). Drift toward party.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>roaming, pursuing, degranulating</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Contact is lethal: 40 HP/sec. Degranulate proteases and ROS in radius. Attack both siderophores and characters. Apoptosis at dawn.</t>
-        </is>
-      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Nocturnal only. All zones. More spawn each night as BBB degrades.</t>
+          <t>Contact is lethal: 40 HP/sec. Degranulate proteases and ROS in radius. Attack both siderophores and characters. Apoptosis at dawn. More spawn each night as BBB degrades.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
+          <t>Nocturnal only. All zones.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>Mandatory shelter at night. Cannot traverse while active. Dawn clears them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Based on mast cells, tissue-resident innate immune sentinels positioned at strategic boundaries (BBB, meninges, thalamus, hypothalamus, hippocampus). Upon activation by pathogens, complement fragments (C3a, C5a), or neuropeptides, they undergo rapid directional degranulation releasing histamine, tryptase, chymase, heparin, TNF-alpha, and serotonin. Mast cell activation amplifies neuroinflammation, increases BBB permeability, and promotes microglial activation.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Kempuraj et al. (2019) Frontiers in Cellular Neuroscience, "Mast Cells in Stress, Pain, Blood-Brain Barrier, Neuroinflammation and Alzheimer's Disease." 13, 54.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Mast_cell</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Watches a cone-shaped zone from fixed position. Does not move.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>idle (watching), charging (~1s visible windup), firing, reloading</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Direct shot along a line after visible charge (swelling, color shift, pressurizing hiss). High damage, narrow spread. Cover (pillars, walls, debris) blocks the shot. Never repositions.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Zone 2-3. Elevated or recessed positions (ledges, grates, wall alcoves).</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Stay out of cone, time movement during reload cycle, use cover between you and the Sentinel.</t>
         </is>
       </c>
     </row>
@@ -1074,15 +1192,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1093,25 +1212,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Real Biology</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Citation</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Mechanic</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Zones</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Clearance</t>
         </is>
@@ -1125,25 +1249,30 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Inflammatory cascade. Immune overreaction flooding tissue with cytokines and reactive molecules.</t>
+          <t>Neuroinflammatory cascades involving self-amplifying feedback loops: activated microglia and astrocytes release TNF-alpha, IL-1beta, IL-6, which further activate neighboring glia, recruit peripheral immune cells via chemokines (CCL2, CXCL10), and compromise BBB integrity. Driven by DAMPs (aggregated amyloid-beta, alpha-synuclein, extracellular ATP) activating microglial NLRP3 inflammasomes and TLR2/4 receptors.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sky darkens. Ambient light amber to pulsing red. Particulate increase. Infrastructure hum to roar. Builds over several in-game minutes.</t>
+          <t>Heneka et al. (2013) Nature, "NLRP3 is activated in Alzheimer's disease and contributes to pathology in APP/PS1 mice." 493(7434), 674–678.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Neuroinflammation</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>HP passive drain. Stamina regen stops. Visibility near-zero. Pathogens scatter. Learnable cycle pattern. Aftermath: corridors reshuffled, fresh iron deposits.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>All zones. Periodic forcing function (like Rain World rain).</t>
-        </is>
-      </c>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>All zones. Periodic forcing function.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Find shelter or environmental seals. Warning phase gives time to prepare.</t>
         </is>
@@ -1157,25 +1286,30 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Microbial biofilm colonization of surfaces.</t>
+          <t>Microbial biofilms are structured communities encased in extracellular polymeric substance (EPS) of polysaccharides, proteins, and eDNA, conferring up to 1000-fold antibiotic resistance. Polymicrobial biofilms including P. gingivalis, spirochetes, and fungi have been detected in AD brain tissue.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Slow terrain patches in unmaintained corridors. Spreads if unaddressed.</t>
+          <t>Kumar et al. (2016) Science Translational Medicine, "Amyloid-beta peptide protects against microbial infection in mouse and worm models of Alzheimer's disease." 8(340), 340ra72.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Reduces movement speed significantly. Drains stamina faster.</t>
+          <t>https://en.wikipedia.org/wiki/Biofilm</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Reduces movement speed significantly. Drains stamina faster. Spreads if unaddressed.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Zone 3 primarily. Everywhere unmaintained.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Peris flora tending, or route around.</t>
         </is>
@@ -1189,25 +1323,30 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Iron accumulation zones (ferritin deposits, free iron saturation).</t>
+          <t>Iron accumulates pathologically in specific brain regions in all major neurodegenerative diseases. Redox-active labile iron (Fe2+) catalyzes Fenton reactions generating hydroxyl radicals. Ferroptosis, an iron-dependent regulated cell death via lipid peroxidation and GPX4 inactivation, links iron dyshomeostasis to neuronal death. Ferritin becomes increasingly iron-loaded and dysfunctional with disease.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Rust-colored particulate, orange-brown discoloration. Visible environmental marker.</t>
+          <t>Stockwell et al. (2017) Cell, "Ferroptosis: A Regulated Cell Death Nexus Linking Metabolism, Redox Biology, and Disease." 171(2), 273–285.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Passive drain on Oli iron reserves. Perception interference (Peris fog creeps faster, Aster data noise spikes). Some cure components hidden inside (risk/reward).</t>
+          <t>https://en.wikipedia.org/wiki/Ferroptosis</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Passive drain on Oli iron reserves. Perception interference (Peris fog, Aster data noise). Some cure components hidden inside (risk/reward). Siderophore reproduction site.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Zone 2-3. Near siderophore feeding grounds.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Oli iron management. Avoid or exploit for resources.</t>
         </is>
@@ -1221,25 +1360,30 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Airborne particulate zones from fungal/microbial sources.</t>
+          <t>Airborne particulate from fungal/microbial sources. Fungal infections of the CNS (Candida, Aspergillus, Cryptococcus) release spores and hyphal fragments that trigger inflammatory responses. Fungal DNA and antigens have been detected in AD brain tissue.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Hazy air with visible particulate. Often near Infiltrator colonies or poorly ventilated areas.</t>
+          <t>Pisa et al. (2015) Scientific Reports, "Different Brain Regions are Infected with Fungi in Alzheimer's Disease." 5, 15015.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Slow stamina regeneration significantly. Devastating if entered with low stamina before real threat. Some cyclic (clear at certain times).</t>
+          <t>https://en.wikipedia.org/wiki/Fungal_meningitis</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Slows stamina regeneration significantly. Some cyclic (clear at certain times). Devastating if entered with low stamina.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Zone 3 primarily. Near Infiltrator colonies.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Wait for clear cycle, or push through with high stamina.</t>
         </is>
@@ -1253,25 +1397,30 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure interference frequencies disrupting cellular processes.</t>
+          <t>Based on excitotoxicity and disrupted neural oscillations in neurodegeneration. Pathological calcium signaling and glutamate excitotoxicity disrupt normal synaptic transmission frequencies, creating zones of aberrant electrical activity. Gamma oscillation disruption (40 Hz) is an early marker of AD.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Audible hum or distortion effect. Entire sub-areas can be resonance zones.</t>
+          <t>Iaccarino et al. (2016) Nature, "Gamma frequency entrainment attenuates amyloid load and modifies microglia." 540(7632), 230–235.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>https://en.wikipedia.org/wiki/Excitotoxicity</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>Increases party ability cooldowns while inside.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Zone 3. Resonance Chambers sub-area is entirely this hazard.</t>
-        </is>
-      </c>
       <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Zone 3. Resonance Chambers sub-area entirely.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Aster hacking can shut down responsible infrastructure.</t>
         </is>
@@ -1288,7 +1437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1539,6 +1688,28 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Corridor traffic</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Fixed-position cone watch with direct shot on detection.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Creates cover-and-sightline gameplay. Forces route planning around known positions.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>